<commit_message>
Escape text in HTML output and keep formula-like text inert in Excel
Plant names, event categories and QC messages can come from user files: the HTML report and the docs page escape them, the embedded JSON cannot close its script element, spreadsheet cells starting with = + - @ are stored as text, and unknown event categories are read as other.
</commit_message>
<xml_diff>
--- a/results/pl_demo/report.xlsx
+++ b/results/pl_demo/report.xlsx
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-132048.309599896</v>
+        <v>-132048.3095998961</v>
       </c>
     </row>
     <row r="11">
@@ -822,16 +822,16 @@
         <v>-0.6218770552512286</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>-24434.16318482063</v>
+        <v>-24434.16318482064</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>-665.105832394442</v>
+        <v>-665.1058323944419</v>
       </c>
       <c r="I2" s="7" t="n">
         <v>-129.7258998352661</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>-72.18467164327956</v>
+        <v>-72.18467164327967</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>-15371.53214130823</v>
@@ -840,7 +840,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>236.1236511742855</v>
+        <v>236.1236511742854</v>
       </c>
       <c r="N2" s="7" t="n">
         <v>0</v>
@@ -886,19 +886,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>78950.2752383558</v>
+        <v>78950.27523835581</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>56808.98189623981</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>-22141.29334211599</v>
+        <v>-22141.29334211601</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>-0.2804460563977775</v>
+        <v>-0.2804460563977777</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>594.867726728243</v>
+        <v>594.8677267282432</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>1530.035544617784</v>
@@ -907,7 +907,7 @@
         <v>-289.4859484915066</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>907.7739631979027</v>
+        <v>907.773963197903</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>-22917.37323981184</v>
@@ -916,7 +916,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>816.0170965778827</v>
+        <v>816.0170965778829</v>
       </c>
       <c r="N3" s="7" t="n">
         <v>0</v>
@@ -925,7 +925,7 @@
         <v>-184.1477989867178</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>-2598.980685947739</v>
+        <v>-2598.980685947754</v>
       </c>
       <c r="Q3" s="7" t="n">
         <v>0</v>
@@ -943,7 +943,7 @@
         <v>0.5728848651876479</v>
       </c>
       <c r="V3" s="6" t="n">
-        <v>0.8485356093850368</v>
+        <v>0.848535609385037</v>
       </c>
       <c r="W3" s="6" t="n">
         <v>1</v>
@@ -1044,28 +1044,28 @@
         <v>163290.611412309</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>2822.770634161367</v>
+        <v>2822.770634161396</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.01759088064295665</v>
+        <v>0.01759088064295683</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>7968.395753944356</v>
+        <v>7968.395753944355</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>2682.94346502555</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>-748.6700268988355</v>
+        <v>-748.6700268988354</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>1309.533602942721</v>
+        <v>1309.53360294272</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>286.5912259636895</v>
+        <v>286.5912259636892</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>-1078.082921911311</v>
@@ -1077,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>-2612.656792203029</v>
+        <v>-2612.656792202996</v>
       </c>
       <c r="Q5" s="7" t="n">
         <v>0</v>
@@ -1086,7 +1086,7 @@
         <v>152.2387239310186</v>
       </c>
       <c r="S5" s="8" t="n">
-        <v>145.1624080586872</v>
+        <v>145.1624080586871</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>0.8125725534965796</v>
@@ -1129,22 +1129,22 @@
         <v>67964.19360628234</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>-1402.184774523771</v>
+        <v>-1402.18477452375</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>-922.9085583037006</v>
+        <v>-922.9085583037007</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>2404.859396495849</v>
+        <v>2404.85939649585</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>739.5176829774903</v>
+        <v>739.5176829774907</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>-593.9700377739598</v>
+        <v>-593.9700377739591</v>
       </c>
       <c r="N6" s="7" t="n">
         <v>-3868.403967154737</v>
@@ -1153,7 +1153,7 @@
         <v>-491.1758709859184</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>-3005.175245824248</v>
+        <v>-3005.175245824292</v>
       </c>
       <c r="Q6" s="7" t="n">
         <v>0</v>
@@ -1266,37 +1266,37 @@
         <v>1</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>193258.4165004726</v>
+        <v>193258.4165004727</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>182781.9321032366</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>-10476.48439723605</v>
+        <v>-10476.48439723608</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>-0.05420971871209776</v>
+        <v>-0.05420971871209791</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>-11265.87365570224</v>
+        <v>-11265.87365570226</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>988.7813743782102</v>
+        <v>988.7813743782508</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>-1028.696613928224</v>
+        <v>-1028.696613928225</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>2011.030109984859</v>
+        <v>2011.03010998486</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>563.4071606013553</v>
+        <v>563.4071606013555</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>1837.905329345662</v>
+        <v>1837.905329345663</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>0</v>
@@ -1305,7 +1305,7 @@
         <v>0</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>-3583.038101915678</v>
+        <v>-3583.038101915729</v>
       </c>
       <c r="Q8" s="7" t="n">
         <v>0</v>
@@ -1323,7 +1323,7 @@
         <v>0.839842317086501</v>
       </c>
       <c r="V8" s="6" t="n">
-        <v>0.8087214927755023</v>
+        <v>0.8087214927755024</v>
       </c>
       <c r="W8" s="6" t="n">
         <v>1</v>
@@ -1348,22 +1348,22 @@
         <v>141746.4848634638</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>-40998.96162535483</v>
+        <v>-40998.96162535486</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>-0.2243501133028963</v>
+        <v>-0.2243501133028964</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>-37027.40227455123</v>
+        <v>-37027.40227455124</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>3127.659777725449</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>-897.2447093138578</v>
+        <v>-897.2447093138579</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>2113.128809403858</v>
+        <v>2113.128809403859</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>0</v>
@@ -1372,7 +1372,7 @@
         <v>142.9195086887162</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>575.4298620669316</v>
+        <v>575.4298620669318</v>
       </c>
       <c r="N9" s="7" t="n">
         <v>-6277.538304255501</v>
@@ -1381,7 +1381,7 @@
         <v>0</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>-2755.914295119197</v>
+        <v>-2755.914295119219</v>
       </c>
       <c r="Q9" s="7" t="n">
         <v>0</v>
@@ -1399,7 +1399,7 @@
         <v>0.8013487335377417</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>0.8109592475346843</v>
+        <v>0.8109592475346846</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>0.9955830388692579</v>
@@ -1475,7 +1475,7 @@
         <v>0.835668114741745</v>
       </c>
       <c r="V10" s="6" t="n">
-        <v>0.841519650797004</v>
+        <v>0.8415196507970039</v>
       </c>
       <c r="W10" s="6" t="n">
         <v>1</v>
@@ -1500,10 +1500,10 @@
         <v>110839.204004973</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>7739.645372560073</v>
+        <v>7739.645372560088</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.0750696266329781</v>
+        <v>0.07506962663297825</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>14637.99728011901</v>
@@ -1512,10 +1512,10 @@
         <v>266.7350286742276</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>-809.0667472756576</v>
+        <v>-809.0667472756575</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>538.8077317768493</v>
+        <v>538.8077317768491</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>0</v>
@@ -1533,7 +1533,7 @@
         <v>-804.3519378389045</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>-2940.986929064735</v>
+        <v>-2940.986929064718</v>
       </c>
       <c r="Q11" s="7" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
         <v>0.7930412300212368</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>0.853574336345421</v>
+        <v>0.8535743363454209</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>0.9793181818181819</v>
@@ -1585,16 +1585,16 @@
         <v>34.51341896116143</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>-9.388119643162433</v>
+        <v>-9.388119643153544</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>-290.3388907443996</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>245.5824475936233</v>
+        <v>245.5824475936234</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>-207.1764658172947</v>
+        <v>-207.1764658172946</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>0</v>
@@ -1609,7 +1609,7 @@
         <v>0</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>-874.1825485832384</v>
+        <v>-874.1825485832475</v>
       </c>
       <c r="Q12" s="7" t="n">
         <v>0</v>
@@ -1694,7 +1694,7 @@
         <v>32.13187524318734</v>
       </c>
       <c r="S13" s="8" t="n">
-        <v>38.44399173156949</v>
+        <v>38.4439917315695</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>0.5099194461257446</v>
@@ -1703,7 +1703,7 @@
         <v>0.4695346894054039</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>0.8539321003949489</v>
+        <v>0.8539321003949488</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>1</v>
@@ -1798,28 +1798,28 @@
         <v>1</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>78950.2752383558</v>
+        <v>78950.27523835581</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>76462.6735725835</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>-2487.601665772294</v>
+        <v>-2487.601665772308</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>-0.03150846096814824</v>
+        <v>-0.03150846096814842</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>-5403.359962463324</v>
+        <v>-5403.359962463326</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>745.6849445887161</v>
+        <v>745.6849445887162</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-636.1720684819981</v>
+        <v>-636.1720684819982</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>964.0096792661432</v>
+        <v>964.0096792661434</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2301.044303405161</v>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>744.0043247676693</v>
+        <v>744.0043247676696</v>
       </c>
       <c r="N15" s="7" t="n">
         <v>0</v>
@@ -1837,7 +1837,7 @@
         <v>0</v>
       </c>
       <c r="P15" s="7" t="n">
-        <v>-1202.812886854661</v>
+        <v>-1202.812886854675</v>
       </c>
       <c r="Q15" s="7" t="n">
         <v>0</v>
@@ -1855,7 +1855,7 @@
         <v>0.8402369313119968</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>0.8485356093850368</v>
+        <v>0.848535609385037</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>1</v>
@@ -1956,28 +1956,28 @@
         <v>149331.537697487</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>-11136.30308066061</v>
+        <v>-11136.30308066058</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>-0.06939897132445957</v>
+        <v>-0.06939897132445941</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>-584.2818915357689</v>
+        <v>-584.2818915357688</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>2655.883147173159</v>
+        <v>2655.883147173158</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>-1519.797481596776</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>2111.072330653802</v>
+        <v>2111.072330653801</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>-1440.824230274726</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>374.1134977619407</v>
+        <v>374.1134977619406</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>-2876.298141245901</v>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="P17" s="7" t="n">
-        <v>-2783.742808081597</v>
+        <v>-2783.742808081566</v>
       </c>
       <c r="Q17" s="7" t="n">
         <v>0</v>
@@ -1998,7 +1998,7 @@
         <v>144.5143633040089</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>145.1624080586872</v>
+        <v>145.1624080586871</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>0.7828284345905447</v>
@@ -2041,19 +2041,19 @@
         <v>82348.43955791164</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>-2751.0266068962</v>
+        <v>-2751.026606896177</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>-2003.184343905372</v>
+        <v>-2003.184343905373</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>309.0443818054355</v>
+        <v>309.0443818054359</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>240.7483239622334</v>
+        <v>240.7483239622336</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-370.8714603967042</v>
@@ -2065,7 +2065,7 @@
         <v>-7387.040093330823</v>
       </c>
       <c r="P18" s="7" t="n">
-        <v>-3891.082158281977</v>
+        <v>-3891.082158281992</v>
       </c>
       <c r="Q18" s="7" t="n">
         <v>0</v>
@@ -2178,19 +2178,19 @@
         <v>1</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>193258.4165004726</v>
+        <v>193258.4165004727</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>179408.6715834</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>-13849.74491707265</v>
+        <v>-13849.74491707268</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>-0.07166438164952456</v>
+        <v>-0.07166438164952471</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>-1517.380422102927</v>
+        <v>-1517.380422102949</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>1254.830317644193</v>
@@ -2205,7 +2205,7 @@
         <v>0</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>535.9815050460344</v>
+        <v>535.9815050460345</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>-7221.160780675358</v>
@@ -2217,7 +2217,7 @@
         <v>-100.4894169134919</v>
       </c>
       <c r="P20" s="7" t="n">
-        <v>-3888.89604036007</v>
+        <v>-3888.896040360079</v>
       </c>
       <c r="Q20" s="7" t="n">
         <v>0</v>
@@ -2235,7 +2235,7 @@
         <v>0.7815695349459229</v>
       </c>
       <c r="V20" s="6" t="n">
-        <v>0.8087214927755023</v>
+        <v>0.8087214927755024</v>
       </c>
       <c r="W20" s="6" t="n">
         <v>0.955818294959552</v>
@@ -2260,16 +2260,16 @@
         <v>173312.4354631724</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>-9433.011025646265</v>
+        <v>-9433.011025646294</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>-0.05161830954963591</v>
+        <v>-0.05161830954963607</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-4602.648457465818</v>
+        <v>-4602.648457465819</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>341.2546240906809</v>
+        <v>341.254624090681</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>-1963.594876763722</v>
@@ -2293,7 +2293,7 @@
         <v>0</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>-4402.883319905093</v>
+        <v>-4402.883319905122</v>
       </c>
       <c r="Q21" s="7" t="n">
         <v>0</v>
@@ -2311,7 +2311,7 @@
         <v>0.8182602461498787</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>0.8109592475346843</v>
+        <v>0.8109592475346846</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
@@ -2387,7 +2387,7 @@
         <v>0.8234529898802112</v>
       </c>
       <c r="V22" s="6" t="n">
-        <v>0.841519650797004</v>
+        <v>0.8415196507970039</v>
       </c>
       <c r="W22" s="6" t="n">
         <v>0.98933281613654</v>
@@ -2412,13 +2412,13 @@
         <v>95883.35271959461</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>-7216.205912818317</v>
+        <v>-7216.205912818303</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>-0.0699925975294103</v>
+        <v>-0.06999259752941017</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-5815.217260650803</v>
+        <v>-5815.217260650802</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>255.2387264133279</v>
@@ -2427,7 +2427,7 @@
         <v>-1152.273859451231</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>737.9590570782096</v>
+        <v>737.9590570782094</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>0</v>
@@ -2436,7 +2436,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="7" t="n">
-        <v>973.6091539265082</v>
+        <v>973.609153926508</v>
       </c>
       <c r="N23" s="7" t="n">
         <v>0</v>
@@ -2445,7 +2445,7 @@
         <v>0</v>
       </c>
       <c r="P23" s="7" t="n">
-        <v>-2215.521730134328</v>
+        <v>-2215.521730134315</v>
       </c>
       <c r="Q23" s="7" t="n">
         <v>0</v>
@@ -2463,7 +2463,7 @@
         <v>0.828214022677109</v>
       </c>
       <c r="V23" s="6" t="n">
-        <v>0.853574336345421</v>
+        <v>0.8535743363454209</v>
       </c>
       <c r="W23" s="6" t="n">
         <v>1</v>
@@ -2497,22 +2497,22 @@
         <v>10862.69655656798</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>66.14677435415042</v>
+        <v>66.14677435416171</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-621.9311774724973</v>
+        <v>-621.9311774724976</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>305.7537485806654</v>
+        <v>305.7537485806657</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>126.0268824931763</v>
+        <v>126.0268824931764</v>
       </c>
       <c r="L24" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M24" s="7" t="n">
-        <v>508.1401301169217</v>
+        <v>508.1401301169218</v>
       </c>
       <c r="N24" s="7" t="n">
         <v>0</v>
@@ -2521,7 +2521,7 @@
         <v>0</v>
       </c>
       <c r="P24" s="7" t="n">
-        <v>-1494.469629975889</v>
+        <v>-1494.469629975902</v>
       </c>
       <c r="Q24" s="7" t="n">
         <v>0</v>
@@ -2606,7 +2606,7 @@
         <v>27.82518587414772</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>38.44399173156949</v>
+        <v>38.4439917315695</v>
       </c>
       <c r="T25" s="6" t="n">
         <v>0.5316159772172223</v>
@@ -2615,7 +2615,7 @@
         <v>0.49034854124502</v>
       </c>
       <c r="V25" s="6" t="n">
-        <v>0.8539321003949489</v>
+        <v>0.8539321003949488</v>
       </c>
       <c r="W25" s="6" t="n">
         <v>1</v>
@@ -2649,10 +2649,10 @@
         <v>-34261.79426377016</v>
       </c>
       <c r="H26" s="7" t="n">
-        <v>-981.4248458116223</v>
+        <v>-981.4248458116222</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-401.5037095515552</v>
+        <v>-401.5037095515551</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>306.4110479108282</v>
@@ -2710,16 +2710,16 @@
         <v>1</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>78950.2752383558</v>
+        <v>78950.27523835581</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>66568.82795554497</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>-12381.44728281083</v>
+        <v>-12381.44728281084</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>-0.1568258913022211</v>
+        <v>-0.1568258913022213</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>-10380.57254371991</v>
@@ -2728,10 +2728,10 @@
         <v>1513.649086180872</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-945.7617943573766</v>
+        <v>-945.7617943573769</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>657.464445195978</v>
+        <v>657.4644451959782</v>
       </c>
       <c r="K27" s="7" t="n">
         <v>-2565.317900860577</v>
@@ -2740,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="7" t="n">
-        <v>698.3594948127217</v>
+        <v>698.3594948127219</v>
       </c>
       <c r="N27" s="7" t="n">
         <v>0</v>
@@ -2749,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="P27" s="7" t="n">
-        <v>-1359.268070062535</v>
+        <v>-1359.268070062548</v>
       </c>
       <c r="Q27" s="7" t="n">
         <v>0</v>
@@ -2767,7 +2767,7 @@
         <v>0.7750621868193456</v>
       </c>
       <c r="V27" s="6" t="n">
-        <v>0.8485356093850368</v>
+        <v>0.848535609385037</v>
       </c>
       <c r="W27" s="6" t="n">
         <v>1</v>
@@ -2868,16 +2868,16 @@
         <v>138842.4589273572</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>-21625.38185079044</v>
+        <v>-21625.38185079041</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>-0.1347645842676246</v>
+        <v>-0.1347645842676244</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>-14798.68215301403</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>2090.473964489261</v>
+        <v>2090.47396448926</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>-2115.794589901617</v>
@@ -2889,10 +2889,10 @@
         <v>0</v>
       </c>
       <c r="L29" s="7" t="n">
-        <v>344.2177471612599</v>
+        <v>344.2177471612598</v>
       </c>
       <c r="M29" s="7" t="n">
-        <v>-3155.477546752737</v>
+        <v>-3155.477546752738</v>
       </c>
       <c r="N29" s="7" t="n">
         <v>-3095.894681552075</v>
@@ -2901,7 +2901,7 @@
         <v>0</v>
       </c>
       <c r="P29" s="7" t="n">
-        <v>-2659.78519562821</v>
+        <v>-2659.785195628185</v>
       </c>
       <c r="Q29" s="7" t="n">
         <v>0</v>
@@ -2910,7 +2910,7 @@
         <v>131.7633171634828</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>145.1624080586872</v>
+        <v>145.1624080586871</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>0.7982774209840894</v>
@@ -2953,7 +2953,7 @@
         <v>81222.54214896049</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>-3227.774231273607</v>
+        <v>-3227.774231273585</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>-3001.033344176297</v>
@@ -2977,7 +2977,7 @@
         <v>-904.2903724565216</v>
       </c>
       <c r="P30" s="7" t="n">
-        <v>-4517.073055747751</v>
+        <v>-4517.07305574778</v>
       </c>
       <c r="Q30" s="7" t="n">
         <v>0</v>
@@ -3041,7 +3041,7 @@
         <v>0</v>
       </c>
       <c r="L31" s="7" t="n">
-        <v>1866.871697025658</v>
+        <v>1866.871697025659</v>
       </c>
       <c r="M31" s="7" t="n">
         <v>2075.648812574698</v>
@@ -3090,19 +3090,19 @@
         <v>1</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>193258.4165004726</v>
+        <v>193258.4165004727</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>188561.8435304497</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>-4696.572970022913</v>
+        <v>-4696.572970022942</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>-0.02430203587025369</v>
+        <v>-0.02430203587025383</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>356.0316931085554</v>
+        <v>356.0316931085126</v>
       </c>
       <c r="H32" s="7" t="n">
         <v>618.0544858027797</v>
@@ -3129,7 +3129,7 @@
         <v>0</v>
       </c>
       <c r="P32" s="7" t="n">
-        <v>-4299.876783028177</v>
+        <v>-4299.876783028163</v>
       </c>
       <c r="Q32" s="7" t="n">
         <v>0</v>
@@ -3147,7 +3147,7 @@
         <v>0.8163134803590477</v>
       </c>
       <c r="V32" s="6" t="n">
-        <v>0.8087214927755023</v>
+        <v>0.8087214927755024</v>
       </c>
       <c r="W32" s="6" t="n">
         <v>0.9993887530562348</v>
@@ -3172,22 +3172,22 @@
         <v>160360.4226700121</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>-22385.02381880651</v>
+        <v>-22385.02381880654</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>-0.122492922526396</v>
+        <v>-0.1224929225263962</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>-18220.13936746102</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>680.0632623992461</v>
+        <v>680.0632623992096</v>
       </c>
       <c r="I33" s="7" t="n">
         <v>-2634.986727400244</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>1704.244149341048</v>
+        <v>1704.244149341047</v>
       </c>
       <c r="K33" s="7" t="n">
         <v>0</v>
@@ -3196,7 +3196,7 @@
         <v>207.0240773017236</v>
       </c>
       <c r="M33" s="7" t="n">
-        <v>1638.950129119937</v>
+        <v>1638.950129119936</v>
       </c>
       <c r="N33" s="7" t="n">
         <v>-2083.998644152797</v>
@@ -3205,7 +3205,7 @@
         <v>0</v>
       </c>
       <c r="P33" s="7" t="n">
-        <v>-3676.180697954405</v>
+        <v>-3676.180697954398</v>
       </c>
       <c r="Q33" s="7" t="n">
         <v>0</v>
@@ -3223,7 +3223,7 @@
         <v>0.817266529398056</v>
       </c>
       <c r="V33" s="6" t="n">
-        <v>0.8109592475346843</v>
+        <v>0.8109592475346846</v>
       </c>
       <c r="W33" s="6" t="n">
         <v>0.9998328877005348</v>
@@ -3299,7 +3299,7 @@
         <v>0.8195721196405991</v>
       </c>
       <c r="V34" s="6" t="n">
-        <v>0.841519650797004</v>
+        <v>0.8415196507970039</v>
       </c>
       <c r="W34" s="6" t="n">
         <v>1</v>
@@ -3324,10 +3324,10 @@
         <v>79750.97882628566</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>-23348.57980612727</v>
+        <v>-23348.57980612725</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>-0.226466341038116</v>
+        <v>-0.2264663410381159</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>-22621.40002616533</v>
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="P35" s="7" t="n">
-        <v>-1046.749201485702</v>
+        <v>-1046.749201485691</v>
       </c>
       <c r="Q35" s="7" t="n">
         <v>0</v>
@@ -3375,7 +3375,7 @@
         <v>0.8265959514122257</v>
       </c>
       <c r="V35" s="6" t="n">
-        <v>0.853574336345421</v>
+        <v>0.8535743363454209</v>
       </c>
       <c r="W35" s="6" t="n">
         <v>1</v>
@@ -3409,13 +3409,13 @@
         <v>13449.41518604703</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>-87.1778564720683</v>
+        <v>-87.17785647205643</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-915.6945722529206</v>
+        <v>-915.6945722529207</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>650.6169722404185</v>
+        <v>650.6169722404186</v>
       </c>
       <c r="K36" s="7" t="n">
         <v>39.38653910759558</v>
@@ -3433,7 +3433,7 @@
         <v>0</v>
       </c>
       <c r="P36" s="7" t="n">
-        <v>-1497.025886351155</v>
+        <v>-1497.025886351166</v>
       </c>
       <c r="Q36" s="7" t="n">
         <v>0</v>
@@ -3518,7 +3518,7 @@
         <v>25.31593270643212</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>38.44399173156949</v>
+        <v>38.4439917315695</v>
       </c>
       <c r="T37" s="6" t="n">
         <v>0.6458202443114597</v>
@@ -3527,7 +3527,7 @@
         <v>0.5991321369041408</v>
       </c>
       <c r="V37" s="6" t="n">
-        <v>0.8539321003949489</v>
+        <v>0.8539321003949488</v>
       </c>
       <c r="W37" s="6" t="n">
         <v>1</v>
@@ -3558,13 +3558,13 @@
         <v>-0.5416078357126632</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>-21277.52196085265</v>
+        <v>-21277.52196085266</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>-931.5835626283142</v>
+        <v>-931.5835626283141</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>-788.8940081099075</v>
+        <v>-788.8940081099074</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>-1322.180927657104</v>
@@ -3585,7 +3585,7 @@
         <v>0</v>
       </c>
       <c r="P38" s="7" t="n">
-        <v>-2413.79631715321</v>
+        <v>-2413.796317153203</v>
       </c>
       <c r="Q38" s="7" t="n">
         <v>0</v>
@@ -3622,37 +3622,37 @@
         <v>1</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>78950.2752383558</v>
+        <v>78950.27523835581</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>48395.44491374225</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>-30554.83032461355</v>
+        <v>-30554.83032461356</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>-0.3870136010592314</v>
+        <v>-0.3870136010592315</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>-31200.35752153355</v>
+        <v>-31200.35752153356</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>213.1198150673857</v>
+        <v>213.1198150673858</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>-884.7961017583441</v>
+        <v>-884.7961017583443</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>317.4345603268299</v>
+        <v>317.4345603268301</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>1312.787801068974</v>
+        <v>1312.787801068975</v>
       </c>
       <c r="L39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M39" s="7" t="n">
-        <v>475.5377922235488</v>
+        <v>475.5377922235489</v>
       </c>
       <c r="N39" s="7" t="n">
         <v>0</v>
@@ -3661,7 +3661,7 @@
         <v>0</v>
       </c>
       <c r="P39" s="7" t="n">
-        <v>-788.5566700083873</v>
+        <v>-788.5566700083946</v>
       </c>
       <c r="Q39" s="7" t="n">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>0.8152268675342172</v>
       </c>
       <c r="V39" s="6" t="n">
-        <v>0.8485356093850368</v>
+        <v>0.848535609385037</v>
       </c>
       <c r="W39" s="6" t="n">
         <v>1</v>
@@ -3780,28 +3780,28 @@
         <v>151300.6423500119</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>-9167.198428135714</v>
+        <v>-9167.198428135685</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>-0.05712794777870592</v>
+        <v>-0.05712794777870575</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>1570.010822861549</v>
+        <v>1570.010822861548</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>248.7556592226223</v>
+        <v>248.7556592226222</v>
       </c>
       <c r="I41" s="7" t="n">
         <v>-3123.179562280908</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>1647.71971231171</v>
+        <v>1647.719712311709</v>
       </c>
       <c r="K41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="L41" s="7" t="n">
-        <v>957.7465663225398</v>
+        <v>957.7465663225397</v>
       </c>
       <c r="M41" s="7" t="n">
         <v>-1814.290463504876</v>
@@ -3813,7 +3813,7 @@
         <v>-611.2618308327158</v>
       </c>
       <c r="P41" s="7" t="n">
-        <v>-3088.596551861654</v>
+        <v>-3088.596551861624</v>
       </c>
       <c r="Q41" s="7" t="n">
         <v>0</v>
@@ -3822,7 +3822,7 @@
         <v>146.4057740771996</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>145.1624080586872</v>
+        <v>145.1624080586871</v>
       </c>
       <c r="T41" s="6" t="n">
         <v>0.782904222681608</v>
@@ -3865,13 +3865,13 @@
         <v>106211.7690900649</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>-7175.919167570736</v>
+        <v>-7175.919167570711</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>-4419.748001634614</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>179.9357677797398</v>
+        <v>179.9357677797402</v>
       </c>
       <c r="K42" s="7" t="n">
         <v>0</v>
@@ -3889,7 +3889,7 @@
         <v>0</v>
       </c>
       <c r="P42" s="7" t="n">
-        <v>-5805.377247052631</v>
+        <v>-5805.37724705266</v>
       </c>
       <c r="Q42" s="7" t="n">
         <v>0</v>
@@ -3953,7 +3953,7 @@
         <v>0</v>
       </c>
       <c r="L43" s="7" t="n">
-        <v>1830.457958691545</v>
+        <v>1830.457958691546</v>
       </c>
       <c r="M43" s="7" t="n">
         <v>1440.419555647448</v>
@@ -4002,25 +4002,25 @@
         <v>1</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>193258.4165004726</v>
+        <v>193258.4165004727</v>
       </c>
       <c r="D44" s="7" t="n">
         <v>192178.5829829284</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>-1079.833517544204</v>
+        <v>-1079.833517544233</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>-0.005587510945695674</v>
+        <v>-0.005587510945695824</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7533.431197281674</v>
+        <v>7533.431197281675</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>97.57707170267626</v>
+        <v>97.57707170267628</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-4111.184931704747</v>
+        <v>-4111.184931704748</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>2502.423631039549</v>
@@ -4029,7 +4029,7 @@
         <v>0</v>
       </c>
       <c r="L44" s="7" t="n">
-        <v>558.6497656185292</v>
+        <v>558.6497656185293</v>
       </c>
       <c r="M44" s="7" t="n">
         <v>1987.658988260126</v>
@@ -4041,7 +4041,7 @@
         <v>-2909.184286843305</v>
       </c>
       <c r="P44" s="7" t="n">
-        <v>-4996.426114293718</v>
+        <v>-4996.426114293747</v>
       </c>
       <c r="Q44" s="7" t="n">
         <v>4.547473508864641e-13</v>
@@ -4059,7 +4059,7 @@
         <v>0.804480033574662</v>
       </c>
       <c r="V44" s="6" t="n">
-        <v>0.8087214927755023</v>
+        <v>0.8087214927755024</v>
       </c>
       <c r="W44" s="6" t="n">
         <v>1</v>
@@ -4084,16 +4084,16 @@
         <v>174784.1978716092</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>-7961.248617209436</v>
+        <v>-7961.248617209465</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>-0.04356468940908221</v>
+        <v>-0.04356468940908236</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>-1769.650003431169</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>131.8482184647352</v>
+        <v>131.848218464695</v>
       </c>
       <c r="I45" s="7" t="n">
         <v>-3781.962351595488</v>
@@ -4117,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>-4611.534783712697</v>
+        <v>-4611.534783712686</v>
       </c>
       <c r="Q45" s="7" t="n">
         <v>0</v>
@@ -4135,7 +4135,7 @@
         <v>0.8132911075580559</v>
       </c>
       <c r="V45" s="6" t="n">
-        <v>0.8109592475346843</v>
+        <v>0.8109592475346846</v>
       </c>
       <c r="W45" s="6" t="n">
         <v>0.9872685185185185</v>
@@ -4211,7 +4211,7 @@
         <v>0.8185206022659632</v>
       </c>
       <c r="V46" s="6" t="n">
-        <v>0.841519650797004</v>
+        <v>0.8415196507970039</v>
       </c>
       <c r="W46" s="6" t="n">
         <v>1</v>
@@ -4236,13 +4236,13 @@
         <v>91516.79921599272</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>-11582.7594164202</v>
+        <v>-11582.75941642019</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>-0.1123453831428795</v>
+        <v>-0.1123453831428794</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>-9119.050340685575</v>
+        <v>-9119.050340685573</v>
       </c>
       <c r="H47" s="7" t="n">
         <v>348.6173166330737</v>
@@ -4251,7 +4251,7 @@
         <v>-2046.960524711629</v>
       </c>
       <c r="J47" s="7" t="n">
-        <v>815.6155200192537</v>
+        <v>815.6155200192535</v>
       </c>
       <c r="K47" s="7" t="n">
         <v>0</v>
@@ -4260,7 +4260,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="7" t="n">
-        <v>932.143081653019</v>
+        <v>932.1430816530188</v>
       </c>
       <c r="N47" s="7" t="n">
         <v>0</v>
@@ -4269,7 +4269,7 @@
         <v>0</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>-2513.124469328344</v>
+        <v>-2513.124469328332</v>
       </c>
       <c r="Q47" s="7" t="n">
         <v>0</v>
@@ -4287,7 +4287,7 @@
         <v>0.8162413771463387</v>
       </c>
       <c r="V47" s="6" t="n">
-        <v>0.853574336345421</v>
+        <v>0.8535743363454209</v>
       </c>
       <c r="W47" s="6" t="n">
         <v>1</v>
@@ -4321,22 +4321,22 @@
         <v>12753.28672905174</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>208.117616121655</v>
+        <v>208.1176161216667</v>
       </c>
       <c r="I48" s="7" t="n">
         <v>-1169.163603451875</v>
       </c>
       <c r="J48" s="7" t="n">
-        <v>1.384260141931804</v>
+        <v>1.384260141932032</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>528.4277264549238</v>
+        <v>528.4277264549239</v>
       </c>
       <c r="L48" s="7" t="n">
         <v>0</v>
       </c>
       <c r="M48" s="7" t="n">
-        <v>523.143449190375</v>
+        <v>523.1434491903751</v>
       </c>
       <c r="N48" s="7" t="n">
         <v>0</v>
@@ -4345,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="P48" s="7" t="n">
-        <v>-1654.633583521929</v>
+        <v>-1654.633583521942</v>
       </c>
       <c r="Q48" s="7" t="n">
         <v>0</v>
@@ -4430,7 +4430,7 @@
         <v>26.96996781427691</v>
       </c>
       <c r="S49" s="8" t="n">
-        <v>38.44399173156949</v>
+        <v>38.4439917315695</v>
       </c>
       <c r="T49" s="6" t="n">
         <v>0.8656653797737279</v>
@@ -4439,7 +4439,7 @@
         <v>0.8054767077668686</v>
       </c>
       <c r="V49" s="6" t="n">
-        <v>0.8539321003949489</v>
+        <v>0.8539321003949488</v>
       </c>
       <c r="W49" s="6" t="n">
         <v>1</v>
@@ -4634,13 +4634,13 @@
         <v>725.1817496979924</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>652.9970780547128</v>
+        <v>652.9970780547127</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>17086.73779966528</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>1715.205658357046</v>
+        <v>1715.205658357045</v>
       </c>
       <c r="F2" s="7" t="n">
         <v>0</v>
@@ -4652,7 +4652,7 @@
         <v>175.5257068314058</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>411.6493580056913</v>
+        <v>411.6493580056912</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>0</v>
@@ -4677,7 +4677,7 @@
         <v>373.3246237159318</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>1281.098586913834</v>
+        <v>1281.098586913835</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>25441.13745603209</v>
@@ -4695,7 +4695,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>816.0170965778827</v>
+        <v>816.0170965778829</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>0</v>
@@ -4781,7 +4781,7 @@
         <v>2798.997164034733</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>1720.914242123423</v>
+        <v>1720.914242123422</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>4985.283672701776</v>
@@ -4806,7 +4806,7 @@
         <v>566.8723423625413</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>2971.73173885839</v>
+        <v>2971.731738858391</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>0</v>
@@ -4818,7 +4818,7 @@
         <v>848.1152916190379</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>1587.632974596528</v>
+        <v>1587.632974596529</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>2529.530883211673</v>
@@ -4892,7 +4892,7 @@
         <v>796.3998735003275</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2807.429983485187</v>
+        <v>2807.429983485188</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>0</v>
@@ -4904,13 +4904,13 @@
         <v>0.6288203598490402</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>564.0359809612042</v>
+        <v>564.0359809612045</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1837.905329345662</v>
+        <v>1837.905329345663</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>0</v>
@@ -4935,7 +4935,7 @@
         <v>165.520308230065</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2278.649117633923</v>
+        <v>2278.649117633924</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>0</v>
@@ -5064,13 +5064,13 @@
         <v>371.7856206709197</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>617.368068264543</v>
+        <v>617.3680682645431</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>612.5814973110113</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>405.4050314937166</v>
+        <v>405.4050314937167</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>0</v>
@@ -5211,7 +5211,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>744.0043247676693</v>
+        <v>744.0043247676696</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>0</v>
@@ -5279,7 +5279,7 @@
         <v>380.7064715329781</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>2491.77880218678</v>
+        <v>2491.778802186779</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>1440.824230274726</v>
@@ -5291,13 +5291,13 @@
         <v>606.5889042323074</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>980.7024019942481</v>
+        <v>980.702401994248</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>4502.759197328612</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>1626.461056082711</v>
+        <v>1626.46105608271</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>7072.427503514744</v>
@@ -5322,7 +5322,7 @@
         <v>2848.092519430963</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>3157.136901236398</v>
+        <v>3157.136901236399</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>0</v>
@@ -5420,7 +5420,7 @@
         <v>55.95632382705764</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>591.937828873092</v>
+        <v>591.9378288730921</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9149.983988856446</v>
@@ -5451,7 +5451,7 @@
         <v>282.4169974371333</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>2718.704792952282</v>
+        <v>2718.704792952283</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>0</v>
@@ -5555,7 +5555,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>973.6091539265082</v>
+        <v>973.609153926508</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>0</v>
@@ -5580,13 +5580,13 @@
         <v>475.8800463999856</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>781.633794980651</v>
+        <v>781.6337949806513</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>387.2459762107846</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>513.2728587039609</v>
+        <v>513.272858703961</v>
       </c>
       <c r="F24" s="7" t="n">
         <v>0</v>
@@ -5598,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>508.1401301169217</v>
+        <v>508.1401301169218</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>0</v>
@@ -5715,7 +5715,7 @@
         <v>4725.192627085487</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>2159.87472622491</v>
+        <v>2159.874726224911</v>
       </c>
       <c r="F27" s="7" t="n">
         <v>0</v>
@@ -5727,7 +5727,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>698.3594948127217</v>
+        <v>698.3594948127219</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>0</v>
@@ -5807,13 +5807,13 @@
         <v>542.8371346155656</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>887.0548817768255</v>
+        <v>887.0548817768254</v>
       </c>
       <c r="H29" s="7" t="n">
         <v>4626.627425537802</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1471.149878785065</v>
+        <v>1471.149878785064</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>3095.894681552075</v>
@@ -5967,7 +5967,7 @@
         <v>799.6066042797071</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>2503.850753620755</v>
+        <v>2503.850753620754</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>0</v>
@@ -5985,7 +5985,7 @@
         <v>3.174958318009836</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>1642.125087437947</v>
+        <v>1642.125087437946</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>2083.998644152797</v>
@@ -6096,7 +6096,7 @@
         <v>164.2616009930328</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>814.8785732334513</v>
+        <v>814.8785732334514</v>
       </c>
       <c r="D36" s="7" t="n">
         <v>495.7170573157042</v>
@@ -6182,7 +6182,7 @@
         <v>2010.92563725343</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>688.7447095963261</v>
+        <v>688.7447095963259</v>
       </c>
       <c r="D38" s="7" t="n">
         <v>11245.83126163243</v>
@@ -6225,13 +6225,13 @@
         <v>429.1316528034464</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>746.5662131302763</v>
+        <v>746.5662131302765</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>157.9476387976702</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>1470.735439866644</v>
+        <v>1470.735439866645</v>
       </c>
       <c r="F39" s="7" t="n">
         <v>0</v>
@@ -6243,7 +6243,7 @@
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>475.5377922235488</v>
+        <v>475.5377922235489</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>0</v>
@@ -6323,7 +6323,7 @@
         <v>11.65040562535908</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>969.3969719478989</v>
+        <v>969.3969719478988</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>3422.00185439327</v>
@@ -6409,7 +6409,7 @@
         <v>198.003944543423</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>2028.461903234968</v>
+        <v>2028.461903234969</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>421.4339816909421</v>
@@ -6440,7 +6440,7 @@
         <v>533.7574776859998</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>3036.181108725548</v>
+        <v>3036.181108725549</v>
       </c>
       <c r="D44" s="7" t="n">
         <v>0</v>
@@ -6452,7 +6452,7 @@
         <v>51.34421468011703</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>609.9939802986462</v>
+        <v>609.9939802986463</v>
       </c>
       <c r="H44" s="7" t="n">
         <v>0</v>
@@ -6587,7 +6587,7 @@
         <v>0</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>932.143081653019</v>
+        <v>932.1430816530188</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>0</v>
@@ -6612,13 +6612,13 @@
         <v>803.3280136472922</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>804.712273789224</v>
+        <v>804.7122737892242</v>
       </c>
       <c r="D48" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>528.4277264549238</v>
+        <v>528.4277264549239</v>
       </c>
       <c r="F48" s="7" t="n">
         <v>0</v>
@@ -6630,7 +6630,7 @@
         <v>0</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>523.143449190375</v>
+        <v>523.1434491903751</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>0</v>

</xml_diff>